<commit_message>
test(xlsx assets): correcy column name
</commit_message>
<xml_diff>
--- a/tests/Bntu.Library.CardGenerator.Infrastructure.Tables.Tests/TestAssets/Xlsx/invalid_date_graduation.xlsx
+++ b/tests/Bntu.Library.CardGenerator.Infrastructure.Tables.Tests/TestAssets/Xlsx/invalid_date_graduation.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\repositories\BNTU-library-card-generator\tests\Bntu.Library.CardGenerator.Infrastructure.Tables.Tests\XlsxExamples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\repositories\BNTU-library-card-generator\tests\Bntu.Library.CardGenerator.Infrastructure.Tables.Tests\TestAssets\Xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96637E1E-0DE4-44D3-B5F6-36042BA59D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{154EB6C3-DF2E-40AD-8382-FE60F26C9227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="92">
   <si>
     <t>#</t>
   </si>
@@ -44,9 +44,6 @@
     <t>Форма обучения</t>
   </si>
   <si>
-    <t>Дата начала обучения</t>
-  </si>
-  <si>
     <t>Дата окончания обучения</t>
   </si>
   <si>
@@ -146,9 +143,6 @@
     <t>девушка</t>
   </si>
   <si>
-    <t>2018-09-01</t>
-  </si>
-  <si>
     <t>2022-06-30</t>
   </si>
   <si>
@@ -315,6 +309,9 @@
   </si>
   <si>
     <t>Пол</t>
+  </si>
+  <si>
+    <t>Год поступления</t>
   </si>
 </sst>
 </file>
@@ -661,103 +658,103 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" t="s">
         <v>86</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>87</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>88</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>89</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>90</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>91</v>
       </c>
-      <c r="H1" t="s">
-        <v>92</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>2</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>3</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>4</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>5</v>
-      </c>
-      <c r="M1" t="s">
-        <v>6</v>
       </c>
       <c r="N1" t="s">
         <v>1</v>
       </c>
       <c r="O1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P1" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q1" t="s">
         <v>9</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>10</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>11</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>12</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>13</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>14</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>15</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>16</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>17</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>18</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>19</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>20</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>21</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>22</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>23</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>24</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>25</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AI1" t="s">
         <v>26</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
@@ -765,73 +762,73 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
         <v>29</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>30</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>31</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>32</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>33</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>34</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2">
+        <v>2018</v>
+      </c>
+      <c r="J2" t="s">
         <v>35</v>
       </c>
-      <c r="I2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J2" t="s">
-        <v>37</v>
-      </c>
       <c r="K2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L2">
         <v>10101</v>
       </c>
       <c r="M2" t="s">
+        <v>36</v>
+      </c>
+      <c r="N2" t="s">
+        <v>37</v>
+      </c>
+      <c r="O2" t="s">
         <v>38</v>
       </c>
-      <c r="N2" t="s">
+      <c r="P2" t="s">
         <v>39</v>
       </c>
-      <c r="O2" t="s">
+      <c r="Q2" t="s">
         <v>40</v>
       </c>
-      <c r="P2" t="s">
+      <c r="R2" t="s">
         <v>41</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="S2" t="s">
         <v>42</v>
       </c>
-      <c r="R2" t="s">
+      <c r="T2" t="s">
         <v>43</v>
       </c>
-      <c r="S2" t="s">
+      <c r="U2" t="s">
         <v>44</v>
       </c>
-      <c r="T2" t="s">
+      <c r="V2" t="s">
         <v>45</v>
       </c>
-      <c r="U2" t="s">
-        <v>46</v>
-      </c>
-      <c r="V2" t="s">
-        <v>47</v>
-      </c>
       <c r="AH2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AJ2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:36" x14ac:dyDescent="0.25">
@@ -839,70 +836,70 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" t="s">
         <v>48</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>49</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>50</v>
       </c>
-      <c r="E3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" t="s">
-        <v>52</v>
-      </c>
       <c r="G3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" t="s">
         <v>34</v>
       </c>
-      <c r="H3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3" t="s">
-        <v>36</v>
+      <c r="I3">
+        <v>2018</v>
       </c>
       <c r="K3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L3">
         <v>20202</v>
       </c>
       <c r="M3" t="s">
+        <v>51</v>
+      </c>
+      <c r="N3" t="s">
+        <v>52</v>
+      </c>
+      <c r="O3" t="s">
         <v>53</v>
       </c>
-      <c r="N3" t="s">
+      <c r="P3" t="s">
         <v>54</v>
       </c>
-      <c r="O3" t="s">
+      <c r="Q3" t="s">
         <v>55</v>
       </c>
-      <c r="P3" t="s">
+      <c r="R3" t="s">
+        <v>41</v>
+      </c>
+      <c r="S3" t="s">
         <v>56</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="T3" t="s">
         <v>57</v>
       </c>
-      <c r="R3" t="s">
-        <v>43</v>
-      </c>
-      <c r="S3" t="s">
+      <c r="U3" t="s">
         <v>58</v>
       </c>
-      <c r="T3" t="s">
+      <c r="V3" t="s">
         <v>59</v>
       </c>
-      <c r="U3" t="s">
-        <v>60</v>
-      </c>
-      <c r="V3" t="s">
-        <v>61</v>
-      </c>
       <c r="AH3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AJ3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.25">
@@ -910,70 +907,70 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" t="s">
         <v>62</v>
       </c>
-      <c r="C4" t="s">
+      <c r="F4" t="s">
         <v>63</v>
       </c>
-      <c r="D4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
         <v>64</v>
       </c>
-      <c r="F4" t="s">
-        <v>65</v>
-      </c>
-      <c r="G4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I4" t="s">
-        <v>36</v>
+      <c r="I4">
+        <v>2018</v>
       </c>
       <c r="J4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L4">
         <v>40404</v>
       </c>
       <c r="M4" t="s">
+        <v>65</v>
+      </c>
+      <c r="N4" t="s">
+        <v>37</v>
+      </c>
+      <c r="O4" t="s">
+        <v>66</v>
+      </c>
+      <c r="P4" t="s">
         <v>67</v>
       </c>
-      <c r="N4" t="s">
-        <v>39</v>
-      </c>
-      <c r="O4" t="s">
+      <c r="Q4" t="s">
         <v>68</v>
       </c>
-      <c r="P4" t="s">
+      <c r="R4" t="s">
+        <v>41</v>
+      </c>
+      <c r="S4" t="s">
         <v>69</v>
       </c>
-      <c r="Q4" t="s">
-        <v>70</v>
-      </c>
-      <c r="R4" t="s">
-        <v>43</v>
-      </c>
-      <c r="S4" t="s">
-        <v>71</v>
-      </c>
       <c r="T4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="U4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="AH4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AJ4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
@@ -981,70 +978,70 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" t="s">
+        <v>71</v>
+      </c>
+      <c r="D5" t="s">
         <v>72</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
         <v>73</v>
       </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>74</v>
       </c>
-      <c r="E5" t="s">
-        <v>75</v>
-      </c>
-      <c r="F5" t="s">
-        <v>76</v>
-      </c>
       <c r="G5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
         <v>34</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5">
+        <v>2018</v>
+      </c>
+      <c r="J5" t="s">
         <v>35</v>
       </c>
-      <c r="I5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J5" t="s">
-        <v>37</v>
-      </c>
       <c r="K5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L5">
         <v>20202</v>
       </c>
       <c r="M5" t="s">
+        <v>75</v>
+      </c>
+      <c r="N5" t="s">
+        <v>37</v>
+      </c>
+      <c r="O5" t="s">
+        <v>76</v>
+      </c>
+      <c r="P5" t="s">
         <v>77</v>
       </c>
-      <c r="N5" t="s">
-        <v>39</v>
-      </c>
-      <c r="O5" t="s">
+      <c r="Q5" t="s">
         <v>78</v>
       </c>
-      <c r="P5" t="s">
+      <c r="R5" t="s">
+        <v>41</v>
+      </c>
+      <c r="S5" t="s">
+        <v>69</v>
+      </c>
+      <c r="T5" t="s">
         <v>79</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="V5" t="s">
         <v>80</v>
       </c>
-      <c r="R5" t="s">
-        <v>43</v>
-      </c>
-      <c r="S5" t="s">
-        <v>71</v>
-      </c>
-      <c r="T5" t="s">
-        <v>81</v>
-      </c>
-      <c r="V5" t="s">
-        <v>82</v>
-      </c>
       <c r="AH5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AJ5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>